<commit_message>
completed n96 n128 result input
</commit_message>
<xml_diff>
--- a/ebdd_cluster/results.xlsx
+++ b/ebdd_cluster/results.xlsx
@@ -5,17 +5,30 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adnan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jjavillo\classes\gems\Geometric-LWE-Estimator\ebdd_cluster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{1CB76914-DD7A-445D-BFD7-7667F7DD8334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{634AE043-A910-4CB7-A08B-7E15486901D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DBF5E9B2-C05D-4253-8A7C-2FE945E9C1DC}"/>
+    <workbookView xWindow="19180" yWindow="900" windowWidth="19150" windowHeight="20640" xr2:uid="{DBF5E9B2-C05D-4253-8A7C-2FE945E9C1DC}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -753,7 +766,7 @@
                     <c:v>4.50419182539998</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.50419182539998</c:v>
+                    <c:v>4.1793347209427267</c:v>
                   </c:pt>
                   <c:pt idx="5">
                     <c:v>3.5899771587017093</c:v>
@@ -789,7 +802,7 @@
                     <c:v>4.50419182539998</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.50419182539998</c:v>
+                    <c:v>4.1793347209427267</c:v>
                   </c:pt>
                   <c:pt idx="5">
                     <c:v>3.5899771587017093</c:v>
@@ -872,7 +885,7 @@
                   <c:v>54.984000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>50</c:v>
+                  <c:v>55.335999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>49.991999999999997</c:v>
@@ -958,7 +971,7 @@
                     <c:v>4.4782139296822345</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.4782139296822345</c:v>
+                    <c:v>4.0607960446357092</c:v>
                   </c:pt>
                   <c:pt idx="5">
                     <c:v>3.5418955377029397</c:v>
@@ -994,7 +1007,7 @@
                     <c:v>4.4782139296822345</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.4782139296822345</c:v>
+                    <c:v>4.0607960446357092</c:v>
                   </c:pt>
                   <c:pt idx="5">
                     <c:v>3.5418955377029397</c:v>
@@ -1077,7 +1090,7 @@
                   <c:v>52.64</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>53</c:v>
+                  <c:v>52.816000000000003</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>47.823999999999998</c:v>
@@ -1156,7 +1169,7 @@
                   <c:v>43.95</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>50</c:v>
+                  <c:v>55.533333333333331</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2533,19 +2546,19 @@
         <v>96</v>
       </c>
       <c r="C6">
-        <v>50</v>
+        <v>55.335999999999999</v>
       </c>
       <c r="D6">
-        <v>4.50419182539998</v>
+        <v>4.1793347209427267</v>
       </c>
       <c r="E6">
         <v>125</v>
       </c>
       <c r="F6">
-        <v>53</v>
+        <v>52.816000000000003</v>
       </c>
       <c r="G6">
-        <v>4.4782139296822345</v>
+        <v>4.0607960446357092</v>
       </c>
       <c r="H6">
         <v>125</v>
@@ -2689,22 +2702,22 @@
         <v>128</v>
       </c>
       <c r="C12">
-        <v>50</v>
+        <v>55.533333333333331</v>
       </c>
       <c r="D12">
-        <v>5</v>
+        <v>3.061908048729812</v>
       </c>
       <c r="E12">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F12">
         <v>54</v>
       </c>
       <c r="G12">
-        <v>5</v>
+        <v>2.8224283329989541</v>
       </c>
       <c r="H12">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added statistics to all csvs and updated results
</commit_message>
<xml_diff>
--- a/ebdd_cluster/results.xlsx
+++ b/ebdd_cluster/results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\adnanben\Geometric-LWE-Estimator\ebdd_cluster\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46A6F25-394C-4366-9E28-8032A0C7B881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{029388FA-2393-419B-A03E-6FB320825595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DBF5E9B2-C05D-4253-8A7C-2FE945E9C1DC}"/>
   </bookViews>
@@ -740,25 +740,25 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>6.0571993528362595</c:v>
+                    <c:v>5.8608928087902266</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>5.2570166444476847</c:v>
+                    <c:v>5.5595660076617799</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>4.8694706077765781</c:v>
+                    <c:v>4.8099359528966446</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>4.50419182539998</c:v>
+                    <c:v>4.6391461950831898</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.1793347209427267</c:v>
+                    <c:v>3.5590321264944156</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>3.5899771587017093</c:v>
+                    <c:v>3.6214771536202659</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.8994311098137837</c:v>
+                    <c:v>2.7754425291281017</c:v>
                   </c:pt>
                   <c:pt idx="7">
                     <c:v>2.8455889217952892</c:v>
@@ -776,25 +776,25 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>6.0571993528362595</c:v>
+                    <c:v>5.8608928087902266</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>5.2570166444476847</c:v>
+                    <c:v>5.5595660076617799</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>4.8694706077765781</c:v>
+                    <c:v>4.8099359528966446</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>4.50419182539998</c:v>
+                    <c:v>4.6391461950831898</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.1793347209427267</c:v>
+                    <c:v>3.5590321264944156</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>3.5899771587017093</c:v>
+                    <c:v>3.6214771536202659</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.8994311098137837</c:v>
+                    <c:v>2.7754425291281017</c:v>
                   </c:pt>
                   <c:pt idx="7">
                     <c:v>2.8455889217952892</c:v>
@@ -859,25 +859,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>36.344000000000001</c:v>
+                  <c:v>36.143999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>44.576000000000001</c:v>
+                  <c:v>43.863999999999997</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>51.984000000000002</c:v>
+                  <c:v>51.96</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>54.984000000000002</c:v>
+                  <c:v>55.136000000000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>55.335999999999999</c:v>
+                  <c:v>55.567999999999998</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>49.991999999999997</c:v>
+                  <c:v>49.768000000000001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>46.588709677419352</c:v>
+                  <c:v>49.333333333333336</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>49.181034482758619</c:v>
@@ -929,25 +929,25 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>5.6251207987029046</c:v>
+                    <c:v>5.6363795288774208</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>4.6394896271033952</c:v>
+                    <c:v>4.4754095145115764</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>4.9001159169962518</c:v>
+                    <c:v>4.5568381794341111</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>4.4782139296822345</c:v>
+                    <c:v>3.5133478198473052</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.0607960446357092</c:v>
+                    <c:v>3.7001830817825314</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>3.5418955377029397</c:v>
+                    <c:v>3.5920521585407728</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.9767194967279416</c:v>
+                    <c:v>2.8198988853635134</c:v>
                   </c:pt>
                   <c:pt idx="7">
                     <c:v>2.954776246229502</c:v>
@@ -965,25 +965,25 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>5.6251207987029046</c:v>
+                    <c:v>5.6363795288774208</c:v>
                   </c:pt>
                   <c:pt idx="1">
-                    <c:v>4.6394896271033952</c:v>
+                    <c:v>4.4754095145115764</c:v>
                   </c:pt>
                   <c:pt idx="2">
-                    <c:v>4.9001159169962518</c:v>
+                    <c:v>4.5568381794341111</c:v>
                   </c:pt>
                   <c:pt idx="3">
-                    <c:v>4.4782139296822345</c:v>
+                    <c:v>3.5133478198473052</c:v>
                   </c:pt>
                   <c:pt idx="4">
-                    <c:v>4.0607960446357092</c:v>
+                    <c:v>3.7001830817825314</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>3.5418955377029397</c:v>
+                    <c:v>3.5920521585407728</c:v>
                   </c:pt>
                   <c:pt idx="6">
-                    <c:v>2.9767194967279416</c:v>
+                    <c:v>2.8198988853635134</c:v>
                   </c:pt>
                   <c:pt idx="7">
                     <c:v>2.954776246229502</c:v>
@@ -1048,25 +1048,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>33.496000000000002</c:v>
+                  <c:v>34.375999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>42.055999999999997</c:v>
+                  <c:v>41.712000000000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>49.192</c:v>
+                  <c:v>49.688000000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>52.64</c:v>
+                  <c:v>53.055999999999997</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>52.816000000000003</c:v>
+                  <c:v>53.223999999999997</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>47.823999999999998</c:v>
+                  <c:v>47.872</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>44.688524590163937</c:v>
+                  <c:v>46.903846153846153</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>46.870370370370374</c:v>
@@ -1110,10 +1110,10 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>5.3840040861797274</c:v>
+                    <c:v>5.6250362006003671</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>3.061908048729812</c:v>
+                    <c:v>3.4263283595413427</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -1125,10 +1125,10 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>5.3840040861797274</c:v>
+                    <c:v>5.6250362006003671</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>3.061908048729812</c:v>
+                    <c:v>3.4263283595413427</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -1187,10 +1187,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>43.95</c:v>
+                  <c:v>36.064</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>55.533333333333331</c:v>
+                  <c:v>55.61643835616438</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1228,10 +1228,10 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>5.4467880443431982</c:v>
+                    <c:v>5.9185111466946125</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>2.8224283329989541</c:v>
+                    <c:v>2.475410991021104</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -1243,10 +1243,10 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="9"/>
                   <c:pt idx="0">
-                    <c:v>5.4467880443431982</c:v>
+                    <c:v>5.9185111466946125</c:v>
                   </c:pt>
                   <c:pt idx="8">
-                    <c:v>2.8224283329989541</c:v>
+                    <c:v>2.475410991021104</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -1269,10 +1269,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>42.65</c:v>
+                  <c:v>34.384</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>54</c:v>
+                  <c:v>54.212765957446805</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2165,16 +2165,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>69850</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>117197</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1473200</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>79097</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>311149</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1492249</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2566,19 +2566,19 @@
         <v>64</v>
       </c>
       <c r="C2">
-        <v>36.344000000000001</v>
+        <v>36.143999999999998</v>
       </c>
       <c r="D2">
-        <v>6.0571993528362595</v>
+        <v>5.8608928087902266</v>
       </c>
       <c r="E2">
         <v>125</v>
       </c>
       <c r="F2">
-        <v>33.496000000000002</v>
+        <v>34.375999999999998</v>
       </c>
       <c r="G2">
-        <v>5.6251207987029046</v>
+        <v>5.6363795288774208</v>
       </c>
       <c r="H2">
         <v>125</v>
@@ -2592,19 +2592,19 @@
         <v>72</v>
       </c>
       <c r="C3">
-        <v>44.576000000000001</v>
+        <v>43.863999999999997</v>
       </c>
       <c r="D3">
-        <v>5.2570166444476847</v>
+        <v>5.5595660076617799</v>
       </c>
       <c r="E3">
         <v>125</v>
       </c>
       <c r="F3">
-        <v>42.055999999999997</v>
+        <v>41.712000000000003</v>
       </c>
       <c r="G3">
-        <v>4.6394896271033952</v>
+        <v>4.4754095145115764</v>
       </c>
       <c r="H3">
         <v>125</v>
@@ -2618,19 +2618,19 @@
         <v>80</v>
       </c>
       <c r="C4">
-        <v>51.984000000000002</v>
+        <v>51.96</v>
       </c>
       <c r="D4">
-        <v>4.8694706077765781</v>
+        <v>4.8099359528966446</v>
       </c>
       <c r="E4">
         <v>125</v>
       </c>
       <c r="F4">
-        <v>49.192</v>
+        <v>49.688000000000002</v>
       </c>
       <c r="G4">
-        <v>4.9001159169962518</v>
+        <v>4.5568381794341111</v>
       </c>
       <c r="H4">
         <v>125</v>
@@ -2644,19 +2644,19 @@
         <v>88</v>
       </c>
       <c r="C5">
-        <v>54.984000000000002</v>
+        <v>55.136000000000003</v>
       </c>
       <c r="D5">
-        <v>4.50419182539998</v>
+        <v>4.6391461950831898</v>
       </c>
       <c r="E5">
         <v>125</v>
       </c>
       <c r="F5">
-        <v>52.64</v>
+        <v>53.055999999999997</v>
       </c>
       <c r="G5">
-        <v>4.4782139296822345</v>
+        <v>3.5133478198473052</v>
       </c>
       <c r="H5">
         <v>125</v>
@@ -2670,19 +2670,19 @@
         <v>96</v>
       </c>
       <c r="C6">
-        <v>55.335999999999999</v>
+        <v>55.567999999999998</v>
       </c>
       <c r="D6">
-        <v>4.1793347209427267</v>
+        <v>3.5590321264944156</v>
       </c>
       <c r="E6">
         <v>125</v>
       </c>
       <c r="F6">
-        <v>52.816000000000003</v>
+        <v>53.223999999999997</v>
       </c>
       <c r="G6">
-        <v>4.0607960446357092</v>
+        <v>3.7001830817825314</v>
       </c>
       <c r="H6">
         <v>125</v>
@@ -2696,19 +2696,19 @@
         <v>104</v>
       </c>
       <c r="C7">
-        <v>49.991999999999997</v>
+        <v>49.768000000000001</v>
       </c>
       <c r="D7">
-        <v>3.5899771587017093</v>
+        <v>3.6214771536202659</v>
       </c>
       <c r="E7">
         <v>125</v>
       </c>
       <c r="F7">
-        <v>47.823999999999998</v>
+        <v>47.872</v>
       </c>
       <c r="G7">
-        <v>3.5418955377029397</v>
+        <v>3.5920521585407728</v>
       </c>
       <c r="H7">
         <v>125</v>
@@ -2722,22 +2722,22 @@
         <v>112</v>
       </c>
       <c r="C8">
-        <v>46.588709677419352</v>
+        <v>49.333333333333336</v>
       </c>
       <c r="D8">
-        <v>2.8994311098137837</v>
+        <v>2.7754425291281017</v>
       </c>
       <c r="E8">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="F8">
-        <v>44.688524590163937</v>
+        <v>46.903846153846153</v>
       </c>
       <c r="G8">
-        <v>2.9767194967279416</v>
+        <v>2.8198988853635134</v>
       </c>
       <c r="H8">
-        <v>122</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -2800,22 +2800,22 @@
         <v>64</v>
       </c>
       <c r="C11">
-        <v>43.95</v>
+        <v>36.064</v>
       </c>
       <c r="D11">
-        <v>5.3840040861797274</v>
+        <v>5.6250362006003671</v>
       </c>
       <c r="E11">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="F11">
-        <v>42.65</v>
+        <v>34.384</v>
       </c>
       <c r="G11">
-        <v>5.4467880443431982</v>
+        <v>5.9185111466946125</v>
       </c>
       <c r="H11">
-        <v>100</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -2882,22 +2882,22 @@
         <v>128</v>
       </c>
       <c r="C19">
-        <v>55.533333333333331</v>
+        <v>55.61643835616438</v>
       </c>
       <c r="D19">
-        <v>3.061908048729812</v>
+        <v>3.4263283595413427</v>
       </c>
       <c r="E19">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="F19">
-        <v>54</v>
+        <v>54.212765957446805</v>
       </c>
       <c r="G19">
-        <v>2.8224283329989541</v>
+        <v>2.475410991021104</v>
       </c>
       <c r="H19">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>